<commit_message>
REV04 Change the desige rule and fixed the errors
</commit_message>
<xml_diff>
--- a/Project Outputs for UZ_D_Inverter/Rev04/BOM_JLC/BOM_JLC_UZ_D_Inverter_Variant_V1_Rev04.xlsx
+++ b/Project Outputs for UZ_D_Inverter/Rev04/BOM_JLC/BOM_JLC_UZ_D_Inverter_Variant_V1_Rev04.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\UltraZohm\uz_d_inverter\Project Outputs for UZ_D_Inverter\Rev04\BOM_JLC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Elsys\uz_d_inverter\Project Outputs for UZ_D_Inverter\Rev04\BOM_JLC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9442442E-C668-4996-85D0-4D1DFD8E67AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{889D558B-3966-406A-A664-2A908B0E6198}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-30828" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{05F3B15F-2541-462D-8F2D-28C3FB828A04}"/>
+    <workbookView xWindow="-22710" yWindow="3495" windowWidth="7530" windowHeight="6015" xr2:uid="{82322282-499E-48ED-8E9F-B47CCC5B5CA5}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM_JLC_UZ_D_Inverter_Variant_V" sheetId="1" r:id="rId1"/>
@@ -691,7 +691,7 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -707,7 +707,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -1022,17 +1022,17 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ECBCC8FB-8D93-4322-BC7E-3CAD1F692DBA}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE272F82-1995-447B-B753-28169EA4102B}">
   <dimension ref="A1:E48"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18.77734375" customWidth="1"/>
-    <col min="2" max="2" width="17.44140625" customWidth="1"/>
-    <col min="3" max="3" width="23.88671875" customWidth="1"/>
-    <col min="4" max="5" width="16.33203125" customWidth="1"/>
+    <col min="1" max="1" width="19" customWidth="1"/>
+    <col min="2" max="2" width="17.5703125" customWidth="1"/>
+    <col min="3" max="3" width="24.28515625" customWidth="1"/>
+    <col min="4" max="5" width="16.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -1049,7 +1049,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>5</v>
       </c>
@@ -1066,7 +1066,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
@@ -1083,7 +1083,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>14</v>
       </c>
@@ -1100,7 +1100,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>19</v>
       </c>
@@ -1117,7 +1117,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -1134,7 +1134,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>28</v>
       </c>
@@ -1151,7 +1151,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>32</v>
       </c>
@@ -1168,7 +1168,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>37</v>
       </c>
@@ -1185,7 +1185,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>41</v>
       </c>
@@ -1202,7 +1202,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>45</v>
       </c>
@@ -1219,7 +1219,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>49</v>
       </c>
@@ -1236,7 +1236,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>52</v>
       </c>
@@ -1253,7 +1253,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>55</v>
       </c>
@@ -1268,7 +1268,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>58</v>
       </c>
@@ -1285,7 +1285,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>63</v>
       </c>
@@ -1302,7 +1302,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>67</v>
       </c>
@@ -1319,7 +1319,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>72</v>
       </c>
@@ -1336,7 +1336,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>76</v>
       </c>
@@ -1353,7 +1353,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>80</v>
       </c>
@@ -1370,7 +1370,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>84</v>
       </c>
@@ -1387,7 +1387,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>88</v>
       </c>
@@ -1404,7 +1404,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>91</v>
       </c>
@@ -1421,7 +1421,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>96</v>
       </c>
@@ -1438,7 +1438,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>100</v>
       </c>
@@ -1455,7 +1455,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>104</v>
       </c>
@@ -1472,7 +1472,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>108</v>
       </c>
@@ -1489,7 +1489,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>113</v>
       </c>
@@ -1506,7 +1506,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>117</v>
       </c>
@@ -1523,7 +1523,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>121</v>
       </c>
@@ -1540,7 +1540,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>125</v>
       </c>
@@ -1557,7 +1557,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>96</v>
       </c>
@@ -1574,7 +1574,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>132</v>
       </c>
@@ -1591,7 +1591,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
         <v>136</v>
       </c>
@@ -1608,7 +1608,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
         <v>140</v>
       </c>
@@ -1625,7 +1625,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
         <v>144</v>
       </c>
@@ -1642,7 +1642,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
         <v>149</v>
       </c>
@@ -1659,7 +1659,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
         <v>153</v>
       </c>
@@ -1676,7 +1676,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
         <v>157</v>
       </c>
@@ -1693,7 +1693,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
         <v>162</v>
       </c>
@@ -1710,7 +1710,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
         <v>166</v>
       </c>
@@ -1727,7 +1727,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
         <v>170</v>
       </c>
@@ -1742,7 +1742,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
         <v>173</v>
       </c>
@@ -1759,7 +1759,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
         <v>177</v>
       </c>
@@ -1776,7 +1776,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
         <v>181</v>
       </c>
@@ -1793,7 +1793,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
         <v>185</v>
       </c>
@@ -1810,7 +1810,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
         <v>189</v>
       </c>
@@ -1827,7 +1827,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
         <v>193</v>
       </c>
@@ -1843,7 +1843,7 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>